<commit_message>
Fill template with Maria Soldevila (A) case; fix contra-asset sign in CF worksheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012nWMFk2orvaisxGrBVUj46
</commit_message>
<xml_diff>
--- a/Accounting/Accounting_Homework_Template.xlsx
+++ b/Accounting/Accounting_Homework_Template.xlsx
@@ -10349,15 +10349,15 @@
         <v>+Δ Accum. depreciation – Buildings</v>
       </c>
       <c r="C17" s="77" t="n">
-        <f aca="false">'Balance Sheet'!E17</f>
-        <v>0</v>
+        <f aca="false">-'Balance Sheet'!E17</f>
+        <v>-0</v>
       </c>
       <c r="D17" s="41"/>
       <c r="E17" s="41"/>
       <c r="F17" s="41"/>
       <c r="G17" s="77" t="n">
         <f aca="false">C17-SUM(D17:F17)</f>
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="H17" s="119"/>
       <c r="J17" s="38" t="s">
@@ -10370,15 +10370,15 @@
         <v>+Δ Accum. depreciation – Furn. &amp; equip.</v>
       </c>
       <c r="C18" s="77" t="n">
-        <f aca="false">'Balance Sheet'!E20</f>
-        <v>0</v>
+        <f aca="false">-'Balance Sheet'!E20</f>
+        <v>-0</v>
       </c>
       <c r="D18" s="41"/>
       <c r="E18" s="41"/>
       <c r="F18" s="41"/>
       <c r="G18" s="77" t="n">
         <f aca="false">C18-SUM(D18:F18)</f>
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="H18" s="119"/>
       <c r="J18" s="42" t="s">
@@ -10391,15 +10391,15 @@
         <v>+Δ Accumulated amortization</v>
       </c>
       <c r="C19" s="77" t="n">
-        <f aca="false">'Balance Sheet'!E23</f>
-        <v>0</v>
+        <f aca="false">-'Balance Sheet'!E23</f>
+        <v>-0</v>
       </c>
       <c r="D19" s="41"/>
       <c r="E19" s="41"/>
       <c r="F19" s="41"/>
       <c r="G19" s="77" t="n">
         <f aca="false">C19-SUM(D19:F19)</f>
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="H19" s="119"/>
       <c r="J19" s="42" t="s">

</xml_diff>